<commit_message>
Fix duplicate worksheet margins in T16a Excel template
</commit_message>
<xml_diff>
--- a/nbv_turniermodi_excel/T16a_9-Spieler-Kalender-Vorlage.xlsx
+++ b/nbv_turniermodi_excel/T16a_9-Spieler-Kalender-Vorlage.xlsx
@@ -1754,7 +1754,6 @@
     <x:mergeCell ref="T13:T15"/>
     <x:mergeCell ref="A17:T17"/>
   </x:mergeCells>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:pageMargins left="0.2" right="0.2" top="0.3" bottom="0.3" header="0.1" footer="0.1"/>
   <x:pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="1"/>
 </x:worksheet>
@@ -3124,7 +3123,6 @@
     <x:mergeCell ref="T16:T18"/>
     <x:mergeCell ref="A20:T20"/>
   </x:mergeCells>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:pageMargins left="0.2" right="0.2" top="0.3" bottom="0.3" header="0.1" footer="0.1"/>
   <x:pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="1"/>
 </x:worksheet>
@@ -4486,7 +4484,6 @@
     <x:mergeCell ref="S1:T1"/>
     <x:mergeCell ref="S2:T2"/>
   </x:mergeCells>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:pageMargins left="0.2" right="0.2" top="0.3" bottom="0.3" header="0.1" footer="0.1"/>
   <x:pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="1"/>
 </x:worksheet>
@@ -5725,7 +5722,6 @@
   <x:mergeCells>
     <x:mergeCell ref="A12:P12"/>
   </x:mergeCells>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:pageMargins left="0.2" right="0.2" top="0.3" bottom="0.3" header="0.1" footer="0.1"/>
   <x:pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="1"/>
 </x:worksheet>
@@ -7304,7 +7300,6 @@
       <x:c r="T45" s="2"/>
     </x:row>
   </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:pageMargins left="0.2" right="0.2" top="0.3" bottom="0.3" header="0.1" footer="0.1"/>
   <x:pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="1"/>
 </x:worksheet>

</xml_diff>